<commit_message>
Add new database files and update grid_france.csv structure for enhanced data analysis
</commit_message>
<xml_diff>
--- a/database/wind_grid_france.xlsx
+++ b/database/wind_grid_france.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,99 +441,140 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>wind_type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>LCOE</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>capacity</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>lon</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DT_m</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>cf_expected</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>project_status</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>rec_weight</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>capacity</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>DT_m</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>lat</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>lon</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Saint-Nazaire</t>
+          <t>Dunkerque</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Pays de la Loire</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>65</v>
+          <t>Hauts-de-France</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>offshore</t>
+        </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>58</v>
       </c>
       <c r="E2" t="n">
-        <v>480</v>
+        <v>600</v>
       </c>
       <c r="F2" t="n">
-        <v>12000</v>
+        <v>51.1</v>
       </c>
       <c r="G2" t="n">
-        <v>47.2</v>
+        <v>2.2</v>
       </c>
       <c r="H2" t="n">
-        <v>-2.5</v>
+        <v>10000</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>operating</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Fécamp</t>
+          <t>Saint-Nazaire</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Normandie</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>70</v>
+          <t>Pays de la Loire</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>offshore</t>
+        </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>63</v>
       </c>
       <c r="E3" t="n">
-        <v>500</v>
+        <v>480</v>
       </c>
       <c r="F3" t="n">
-        <v>15000</v>
+        <v>47.2</v>
       </c>
       <c r="G3" t="n">
-        <v>49.8</v>
+        <v>-2.5</v>
       </c>
       <c r="H3" t="n">
-        <v>0.5</v>
+        <v>12000</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>operating</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Courseulles-sur-Mer</t>
+          <t>Fécamp</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -541,89 +582,128 @@
           <t>Normandie</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>72</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>offshore</t>
+        </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>68</v>
       </c>
       <c r="E4" t="n">
-        <v>450</v>
+        <v>500</v>
       </c>
       <c r="F4" t="n">
-        <v>10000</v>
+        <v>49.8</v>
       </c>
       <c r="G4" t="n">
-        <v>49.4</v>
+        <v>0.5</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.5</v>
+        <v>15000</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>operating</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Saint-Brieuc</t>
+          <t>Courseulles-sur-Mer</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bretagne</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>75</v>
+          <t>Normandie</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>offshore</t>
+        </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="E5" t="n">
-        <v>496</v>
+        <v>450</v>
       </c>
       <c r="F5" t="n">
-        <v>16000</v>
+        <v>49.4</v>
       </c>
       <c r="G5" t="n">
-        <v>48.6</v>
+        <v>-0.5</v>
       </c>
       <c r="H5" t="n">
-        <v>-2.8</v>
+        <v>10000</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>construction</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dunkerque</t>
+          <t>Saint-Brieuc</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hauts-de-France</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>60</v>
+          <t>Bretagne</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>offshore</t>
+        </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>72</v>
       </c>
       <c r="E6" t="n">
-        <v>600</v>
+        <v>496</v>
       </c>
       <c r="F6" t="n">
-        <v>10000</v>
+        <v>48.6</v>
       </c>
       <c r="G6" t="n">
-        <v>51.1</v>
+        <v>-2.8</v>
       </c>
       <c r="H6" t="n">
-        <v>2.2</v>
+        <v>16000</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>operating</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Golfe du Lion</t>
+          <t>Golfe du Lion Flottant</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -631,23 +711,294 @@
           <t>Occitanie</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>80</v>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>offshore_floating</t>
+        </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>95</v>
       </c>
       <c r="E7" t="n">
         <v>250</v>
       </c>
       <c r="F7" t="n">
+        <v>43.1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="H7" t="n">
         <v>20000</v>
       </c>
-      <c r="G7" t="n">
-        <v>43.1</v>
-      </c>
-      <c r="H7" t="n">
-        <v>4.2</v>
+      <c r="I7" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Parc HdF Nord</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Hauts-de-France</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>onshore</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>55</v>
+      </c>
+      <c r="E8" t="n">
+        <v>120</v>
+      </c>
+      <c r="F8" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>operating</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Parc Normandie Côtier</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Normandie</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>onshore</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>57</v>
+      </c>
+      <c r="E9" t="n">
+        <v>90</v>
+      </c>
+      <c r="F9" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H9" t="n">
+        <v>8000</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>operating</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Parc Bretagne Centrale</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Bretagne</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>onshore</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>58</v>
+      </c>
+      <c r="E10" t="n">
+        <v>75</v>
+      </c>
+      <c r="F10" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-3</v>
+      </c>
+      <c r="H10" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>operating</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Parc Pays de la Loire</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Pays de la Loire</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>onshore</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>56</v>
+      </c>
+      <c r="E11" t="n">
+        <v>100</v>
+      </c>
+      <c r="F11" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>12000</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>operating</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Parc Occitanie</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Occitanie</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>onshore</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>60</v>
+      </c>
+      <c r="E12" t="n">
+        <v>80</v>
+      </c>
+      <c r="F12" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="G12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" t="n">
+        <v>15000</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>operating</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Parc Grand Est</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Grand Est</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>onshore</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>54</v>
+      </c>
+      <c r="E13" t="n">
+        <v>110</v>
+      </c>
+      <c r="F13" t="n">
+        <v>49</v>
+      </c>
+      <c r="G13" t="n">
+        <v>6</v>
+      </c>
+      <c r="H13" t="n">
+        <v>7000</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>operating</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove obsolete database files and add initial test notebook for solar patterns
</commit_message>
<xml_diff>
--- a/database/wind_grid_france.xlsx
+++ b/database/wind_grid_france.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>